<commit_message>
update ISV analysis and add logging print
</commit_message>
<xml_diff>
--- a/contracts/ChainSwap/output_debug/callPriArgs.xlsx
+++ b/contracts/ChainSwap/output_debug/callPriArgs.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C38"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,6 +444,11 @@
           <t>blockID</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>function</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -461,6 +466,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -478,6 +488,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -495,6 +510,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -512,6 +532,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -529,6 +554,11 @@
           <t>0x140c</t>
         </is>
       </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>0x1348</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -546,6 +576,11 @@
           <t>0x1455</t>
         </is>
       </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0x1348</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -563,6 +598,11 @@
           <t>0x1c5b</t>
         </is>
       </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>0x1c5b</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -580,6 +620,11 @@
           <t>0x1c5b</t>
         </is>
       </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>0x1c5b</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -597,6 +642,11 @@
           <t>0x1c5b</t>
         </is>
       </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>0x1c5b</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -614,6 +664,11 @@
           <t>0x1fdc</t>
         </is>
       </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>0x1d9a</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -631,6 +686,11 @@
           <t>0x1fdc</t>
         </is>
       </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>0x1d9a</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -648,6 +708,11 @@
           <t>0x2024</t>
         </is>
       </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>0x1d9a</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -665,6 +730,11 @@
           <t>0x2024</t>
         </is>
       </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>0x1d9a</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -682,6 +752,11 @@
           <t>0x2037</t>
         </is>
       </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0x2037</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -699,6 +774,11 @@
           <t>0x310cB0x2686B0x2bf4B0x1d11B0x1a19</t>
         </is>
       </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>0x1a19</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -716,6 +796,11 @@
           <t>0x310cB0x2686B0x2c2bB0x1de4B0x1cb8</t>
         </is>
       </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>0x1cb8</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -733,6 +818,11 @@
           <t>0x70f</t>
         </is>
       </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -750,6 +840,11 @@
           <t>0x70f</t>
         </is>
       </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -767,6 +862,11 @@
           <t>0x840</t>
         </is>
       </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -784,6 +884,11 @@
           <t>0x1a0e</t>
         </is>
       </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>0x172c</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -801,6 +906,11 @@
           <t>0x1a68</t>
         </is>
       </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>0x1a19</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -818,6 +928,11 @@
           <t>0x1ca6</t>
         </is>
       </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0x1c5b</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -835,6 +950,11 @@
           <t>0x1d05</t>
         </is>
       </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>0x1cb8</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -852,6 +972,11 @@
           <t>0x1ddc</t>
         </is>
       </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>0x1d9a</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -869,6 +994,11 @@
           <t>0x3c484</t>
         </is>
       </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>0x1348</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -886,6 +1016,11 @@
           <t>0x3c4a8</t>
         </is>
       </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>0x1a83</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -903,6 +1038,11 @@
           <t>0x3c4ef</t>
         </is>
       </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>0x2037</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -920,6 +1060,11 @@
           <t>0x3c560</t>
         </is>
       </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>0x1348</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -937,6 +1082,11 @@
           <t>0x3c584</t>
         </is>
       </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>0x1a83</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -954,6 +1104,11 @@
           <t>0x3c5cb</t>
         </is>
       </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>0x2037</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -971,6 +1126,11 @@
           <t>0x840</t>
         </is>
       </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -988,6 +1148,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1005,6 +1170,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1022,6 +1192,11 @@
           <t>0x719</t>
         </is>
       </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1039,6 +1214,11 @@
           <t>0x2b76B0x2f89B0x719</t>
         </is>
       </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>0x705</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1056,6 +1236,11 @@
           <t>0x2b76B0x2c16B0x1d11B0x1a19</t>
         </is>
       </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>0x1a19</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1071,6 +1256,11 @@
       <c r="C38" t="inlineStr">
         <is>
           <t>0x2b76B0x2c40B0x1de4B0x1cb8</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>0x1cb8</t>
         </is>
       </c>
     </row>

</xml_diff>